<commit_message>
criado rateio de agua entre inquilinos
</commit_message>
<xml_diff>
--- a/outputs/cronograma-aplicacao-alugueis.xlsx
+++ b/outputs/cronograma-aplicacao-alugueis.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="205">
   <si>
     <t xml:space="preserve">Cronograma de Desenvolvimento - Aplicacao de Alugueis</t>
   </si>
@@ -219,7 +219,7 @@
     <t xml:space="preserve">Fase 9</t>
   </si>
   <si>
-    <t xml:space="preserve">Modelo marketplace/split por recebedor, credenciais sandbox. Teste contra o ambiente real do Mercado Pago ainda pendente (ver Riscos).</t>
+    <t xml:space="preserve">Modelo marketplace/split por recebedor. Sandbox do Mercado Pago se mostrou instavel para esse modelo (varios erros: client_id/secret, contas de teste, "Invalid users involved"); validado com um pagamento Pix real de R$1 em producao (ver Fase 20). Recomenda-se mais alguns testes reais de baixo valor antes do uso pleno (ver Riscos).</t>
   </si>
   <si>
     <t xml:space="preserve">Webhooks e conciliacao</t>
@@ -231,7 +231,7 @@
     <t xml:space="preserve">Fase 10</t>
   </si>
   <si>
-    <t xml:space="preserve">Validacao HMAC do webhook e checagem de external_id antes de gravar pagamento.</t>
+    <t xml:space="preserve">Validacao HMAC do webhook e checagem de external_id antes de gravar pagamento. Adicionado tambem um fallback manual: botao admin "Verificar pagamento" que reconcilia a cobranca direto na API da MP quando o webhook nao chega (ver Fase 20).</t>
   </si>
   <si>
     <t xml:space="preserve">Geracao de cobranca mensal (manual e automatica)</t>
@@ -297,7 +297,7 @@
     <t xml:space="preserve">Fases 9 e 13</t>
   </si>
   <si>
-    <t xml:space="preserve">Decisao ja tomada: n8n como orquestrador e WAHA como gateway WhatsApp. Implementacao do envio ainda nao iniciada.</t>
+    <t xml:space="preserve">Decisao revisada em 11/07/2026: Cron Trigger da Cloudflare chama o WAHA diretamente, sem n8n como orquestrador (ver docs/INTEGRACAO_WHATSAPP_WAHA.md). Regua definida (5 dias antes, no vencimento, a cada 3 dias em atraso, confirmacao de pagamento). Implementacao do envio ainda nao iniciada.</t>
   </si>
   <si>
     <t xml:space="preserve">Autoatendimento de senha e gestao de cobrancas</t>
@@ -327,6 +327,51 @@
     <t xml:space="preserve">Inclui teste real do fluxo Pix/Mercado Pago em sandbox e teste de ponta a ponta da aplicacao publicada.</t>
   </si>
   <si>
+    <t xml:space="preserve">Vistoria fotografica e registro de ocorrencias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fotos da vistoria embutidas no PDF do contrato gerado; inquilino registra ocorrencias com fotos e acompanha status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fora do MVP original, adicionado por solicitacao explicita. Fotos da vistoria (camera ou galeria) sao embutidas diretamente no PDF gerado do contrato via pdf-lib, para resguardo em caso de disputa. Inquilino pode reportar ocorrencia (fotos + descricao) e o admin acompanha com status aberta/em analise/resolvida.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teste real do fluxo Pix e comprovante de pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validacao ponta a ponta do Pix (OAuth, cobranca, webhook) e recibo de pagamento em PDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fases 10 e 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrigidos no caminho: client_secret errado (nao e o Access Token), e-mail de login do inquilino que nao sincronizava ao editar, CPF ausente no payload do Pix (obrigatorio pela MP). Webhook de producao nao estava configurado a tempo do primeiro pagamento; adicionado o botao admin "Verificar pagamento" como fallback. Recibo de pagamento em PDF (texto fixo por enquanto) liberado ao inquilino apos a cobranca ser paga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rateio de agua entre imoveis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin informa a fatura de agua do mes, seleciona os imoveis participantes e o valor e somado na cobranca de cada um</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opcional, adicionado por solicitacao explicita (caso de uso: predio com multiplos apartamentos do mesmo dono). Divisao igual entre os imoveis selecionados; fatura de agua (JPG/PNG/PDF) pode ser anexada; valor e somado automaticamente na cobranca do mes (na hora, se ja existir, ou quando a cobranca for gerada).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajustes de responsividade mobile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisao e correcoes de UX para uso em celular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabela de contratos (admin) ganhou menu de acoes compacto no celular (antes exigia rolagem horizontal por 4 botoes lado a lado). Corrigido botao de remover foto de vistoria que dependia de :hover, invisivel em telas touch.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumo Executivo do Projeto</t>
   </si>
   <si>
@@ -369,7 +414,7 @@
     <t xml:space="preserve">Define se o pagamento vai para conta central, multiplas contas ou split</t>
   </si>
   <si>
-    <t xml:space="preserve">Definido: OAuth por recebedor (marketplace/split), sandbox</t>
+    <t xml:space="preserve">Definido: OAuth por recebedor (marketplace/split). Sandbox instavel para esse modelo; validado com pagamento Pix real de R$1 (ver Fase 20)</t>
   </si>
   <si>
     <t xml:space="preserve">Stack do projeto</t>
@@ -390,7 +435,7 @@
     <t xml:space="preserve">Fase 16</t>
   </si>
   <si>
-    <t xml:space="preserve">Definido: n8n + WAHA (implementacao pendente)</t>
+    <t xml:space="preserve">Definido (revisado 11/07/2026): Cron Trigger da Cloudflare chama o WAHA direto, sem n8n; implementacao do envio pendente</t>
   </si>
   <si>
     <t xml:space="preserve">Armazenamento de PDF assinado</t>
@@ -447,7 +492,7 @@
     <t xml:space="preserve">Geracao manual e automatica via cron entregues</t>
   </si>
   <si>
-    <t xml:space="preserve">OAuth por recebedor; teste em sandbox real pendente</t>
+    <t xml:space="preserve">OAuth por recebedor; validado com pagamento Pix real (sandbox instavel para esse modelo)</t>
   </si>
   <si>
     <t xml:space="preserve">Sim (alem do MVP)</t>
@@ -465,7 +510,7 @@
     <t xml:space="preserve">Nao</t>
   </si>
   <si>
-    <t xml:space="preserve">Decisao tomada (n8n+WAHA), implementacao pendente</t>
+    <t xml:space="preserve">Decisao tomada (Cron Trigger + WAHA direto, sem n8n); implementacao pendente</t>
   </si>
   <si>
     <t xml:space="preserve">Depois</t>
@@ -474,6 +519,21 @@
     <t xml:space="preserve">Pode ficar para fase posterior</t>
   </si>
   <si>
+    <t xml:space="preserve">Fotos da vistoria no PDF do contrato; inquilino reporta ocorrencias com fotos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recibo de pagamento (PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liberado ao inquilino apos a cobranca ser paga; texto fixo por enquanto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sim (opcional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divisao igual entre imoveis selecionados; fatura anexavel; soma automatica na cobranca</t>
+  </si>
+  <si>
     <t xml:space="preserve">Riscos e Mitigacoes</t>
   </si>
   <si>
@@ -492,58 +552,58 @@
     <t xml:space="preserve">Alto</t>
   </si>
   <si>
-    <t xml:space="preserve">Fluxo Pix/Mercado Pago nao testado no sandbox real</t>
+    <t xml:space="preserve">Fluxo Pix/Mercado Pago nao validado ponta a ponta</t>
   </si>
   <si>
     <t xml:space="preserve">Falha so seria descoberta em producao, com impacto em recebimento</t>
   </si>
   <si>
-    <t xml:space="preserve">Executar teste completo (OAuth, criacao de cobranca, webhook) no sandbox do Mercado Pago antes do lancamento</t>
+    <t xml:space="preserve">Sandbox da MP se mostrou instavel para o modelo marketplace/OAuth (varios erros ao longo do teste). Validado em vez disso com um pagamento Pix real de R$1, confirmando OAuth, criacao de cobranca, webhook (com fallback manual "Verificar pagamento") e recibo de pagamento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitigado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Webhook duplicado ou perdido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobranca pode ficar com status incorreto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Processamento idempotente por external_id ja implementado; manter logs e reprocessamento manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permissoes mal separadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recebedor ou inquilino pode ver dados indevidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">requireApiUser/requireUser ja aplicados a todas as rotas; manter testes de autorizacao por perfil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculo incorreto de juros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobranca indevida ou perda financeira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adicionar testes automatizados para multa, juros, carencia e abonos</t>
   </si>
   <si>
     <t xml:space="preserve">Aberto</t>
   </si>
   <si>
-    <t xml:space="preserve">Webhook duplicado ou perdido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cobranca pode ficar com status incorreto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Processamento idempotente por external_id ja implementado; manter logs e reprocessamento manual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitigado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Permissoes mal separadas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recebedor ou inquilino pode ver dados indevidos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">requireApiUser/requireUser ja aplicados a todas as rotas; manter testes de autorizacao por perfil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculo incorreto de juros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cobranca indevida ou perda financeira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adicionar testes automatizados para multa, juros, carencia e abonos</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mensagens WhatsApp duplicadas</t>
   </si>
   <si>
     <t xml:space="preserve">Experiencia ruim para o inquilino</t>
   </si>
   <si>
-    <t xml:space="preserve">Controlar envio por cobranca, evento e data quando a integracao n8n/WAHA for implementada</t>
+    <t xml:space="preserve">Controlar envio por cobranca, evento e data quando a integracao Cron Trigger + WAHA (sem n8n, decisao de 11/07/2026) for implementada</t>
   </si>
   <si>
     <t xml:space="preserve">Aberto (fase nao iniciada)</t>
@@ -568,6 +628,15 @@
   </si>
   <si>
     <t xml:space="preserve">Realizar bateria de testes manuais (ou via navegador) cobrindo os fluxos criticos antes do lancamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apenas uma transacao Pix real (R$1) foi validada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Casos de borda (expiracao do QR, estorno, pagamento parcial) ainda nao testados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realizar mais alguns testes reais de baixo valor cobrindo expiracao e falha antes do uso pleno</t>
   </si>
 </sst>
 </file>
@@ -739,8 +808,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -764,7 +837,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1028,1413 +1101,1577 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U22"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="14" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="14" style="1" width="6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U3" s="2" t="s">
+      <c r="U3" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <v>46201</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5" t="n">
         <v>46207</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="6" t="n">
         <f aca="false">ROUNDUP((E4-D4+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="M4" s="6"/>
-      <c r="N4" s="7" t="n">
+      <c r="M4" s="7"/>
+      <c r="N4" s="8" t="n">
         <v>46201</v>
       </c>
-      <c r="O4" s="7" t="n">
+      <c r="O4" s="8" t="n">
         <v>46208</v>
       </c>
-      <c r="P4" s="7" t="n">
+      <c r="P4" s="8" t="n">
         <v>46215</v>
       </c>
-      <c r="Q4" s="7" t="n">
+      <c r="Q4" s="8" t="n">
         <v>46222</v>
       </c>
-      <c r="R4" s="7" t="n">
+      <c r="R4" s="8" t="n">
         <v>46229</v>
       </c>
-      <c r="S4" s="7" t="n">
+      <c r="S4" s="8" t="n">
         <v>46236</v>
       </c>
-      <c r="T4" s="7" t="n">
+      <c r="T4" s="8" t="n">
         <v>46243</v>
       </c>
-      <c r="U4" s="7" t="n">
+      <c r="U4" s="8" t="n">
         <v>46250</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="6" t="n">
         <f aca="false">ROUNDUP((E5-D5+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M5" s="0" t="s">
+      <c r="M5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="N5" s="8" t="str">
+      <c r="N5" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D5,N$4&lt;=$E5),"x","")</f>
         <v/>
       </c>
-      <c r="O5" s="8" t="str">
+      <c r="O5" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D5,O$4&lt;=$E5),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P5" s="8" t="str">
+      <c r="P5" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D5,P$4&lt;=$E5),"x","")</f>
         <v/>
       </c>
-      <c r="Q5" s="8" t="str">
+      <c r="Q5" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D5,Q$4&lt;=$E5),"x","")</f>
         <v/>
       </c>
-      <c r="R5" s="8" t="str">
+      <c r="R5" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D5,R$4&lt;=$E5),"x","")</f>
         <v/>
       </c>
-      <c r="S5" s="8" t="str">
+      <c r="S5" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D5,S$4&lt;=$E5),"x","")</f>
         <v/>
       </c>
-      <c r="T5" s="8" t="str">
+      <c r="T5" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D5,T$4&lt;=$E5),"x","")</f>
         <v/>
       </c>
-      <c r="U5" s="8" t="str">
+      <c r="U5" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D5,U$4&lt;=$E5),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="6" t="n">
         <f aca="false">ROUNDUP((E6-D6+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="M6" s="0" t="s">
+      <c r="M6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N6" s="8" t="str">
+      <c r="N6" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D6,N$4&lt;=$E6),"x","")</f>
         <v/>
       </c>
-      <c r="O6" s="8" t="str">
+      <c r="O6" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D6,O$4&lt;=$E6),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P6" s="8" t="str">
+      <c r="P6" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D6,P$4&lt;=$E6),"x","")</f>
         <v/>
       </c>
-      <c r="Q6" s="8" t="str">
+      <c r="Q6" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D6,Q$4&lt;=$E6),"x","")</f>
         <v/>
       </c>
-      <c r="R6" s="8" t="str">
+      <c r="R6" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D6,R$4&lt;=$E6),"x","")</f>
         <v/>
       </c>
-      <c r="S6" s="8" t="str">
+      <c r="S6" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D6,S$4&lt;=$E6),"x","")</f>
         <v/>
       </c>
-      <c r="T6" s="8" t="str">
+      <c r="T6" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D6,T$4&lt;=$E6),"x","")</f>
         <v/>
       </c>
-      <c r="U6" s="8" t="str">
+      <c r="U6" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D6,U$4&lt;=$E6),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="6" t="n">
         <f aca="false">ROUNDUP((E7-D7+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="M7" s="0" t="s">
+      <c r="M7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="N7" s="8" t="str">
+      <c r="N7" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D7,N$4&lt;=$E7),"x","")</f>
         <v/>
       </c>
-      <c r="O7" s="8" t="str">
+      <c r="O7" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D7,O$4&lt;=$E7),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P7" s="8" t="str">
+      <c r="P7" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D7,P$4&lt;=$E7),"x","")</f>
         <v/>
       </c>
-      <c r="Q7" s="8" t="str">
+      <c r="Q7" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D7,Q$4&lt;=$E7),"x","")</f>
         <v/>
       </c>
-      <c r="R7" s="8" t="str">
+      <c r="R7" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D7,R$4&lt;=$E7),"x","")</f>
         <v/>
       </c>
-      <c r="S7" s="8" t="str">
+      <c r="S7" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D7,S$4&lt;=$E7),"x","")</f>
         <v/>
       </c>
-      <c r="T7" s="8" t="str">
+      <c r="T7" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D7,T$4&lt;=$E7),"x","")</f>
         <v/>
       </c>
-      <c r="U7" s="8" t="str">
+      <c r="U7" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D7,U$4&lt;=$E7),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="6" t="n">
         <f aca="false">ROUNDUP((E8-D8+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="K8" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="M8" s="0" t="s">
+      <c r="M8" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="N8" s="8" t="str">
+      <c r="N8" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D8,N$4&lt;=$E8),"x","")</f>
         <v/>
       </c>
-      <c r="O8" s="8" t="str">
+      <c r="O8" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D8,O$4&lt;=$E8),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P8" s="8" t="str">
+      <c r="P8" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D8,P$4&lt;=$E8),"x","")</f>
         <v/>
       </c>
-      <c r="Q8" s="8" t="str">
+      <c r="Q8" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D8,Q$4&lt;=$E8),"x","")</f>
         <v/>
       </c>
-      <c r="R8" s="8" t="str">
+      <c r="R8" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D8,R$4&lt;=$E8),"x","")</f>
         <v/>
       </c>
-      <c r="S8" s="8" t="str">
+      <c r="S8" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D8,S$4&lt;=$E8),"x","")</f>
         <v/>
       </c>
-      <c r="T8" s="8" t="str">
+      <c r="T8" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D8,T$4&lt;=$E8),"x","")</f>
         <v/>
       </c>
-      <c r="U8" s="8" t="str">
+      <c r="U8" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D8,U$4&lt;=$E8),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="6" t="n">
         <f aca="false">ROUNDUP((E9-D9+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="J9" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="K9" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="M9" s="0" t="s">
+      <c r="M9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="N9" s="8" t="str">
+      <c r="N9" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D9,N$4&lt;=$E9),"x","")</f>
         <v/>
       </c>
-      <c r="O9" s="8" t="str">
+      <c r="O9" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D9,O$4&lt;=$E9),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P9" s="8" t="str">
+      <c r="P9" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D9,P$4&lt;=$E9),"x","")</f>
         <v/>
       </c>
-      <c r="Q9" s="8" t="str">
+      <c r="Q9" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D9,Q$4&lt;=$E9),"x","")</f>
         <v/>
       </c>
-      <c r="R9" s="8" t="str">
+      <c r="R9" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D9,R$4&lt;=$E9),"x","")</f>
         <v/>
       </c>
-      <c r="S9" s="8" t="str">
+      <c r="S9" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D9,S$4&lt;=$E9),"x","")</f>
         <v/>
       </c>
-      <c r="T9" s="8" t="str">
+      <c r="T9" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D9,T$4&lt;=$E9),"x","")</f>
         <v/>
       </c>
-      <c r="U9" s="8" t="str">
+      <c r="U9" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D9,U$4&lt;=$E9),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="6" t="n">
         <f aca="false">ROUNDUP((E10-D10+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="J10" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="K10" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="M10" s="0" t="s">
+      <c r="M10" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="N10" s="8" t="str">
+      <c r="N10" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D10,N$4&lt;=$E10),"x","")</f>
         <v/>
       </c>
-      <c r="O10" s="8" t="str">
+      <c r="O10" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D10,O$4&lt;=$E10),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P10" s="8" t="str">
+      <c r="P10" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D10,P$4&lt;=$E10),"x","")</f>
         <v/>
       </c>
-      <c r="Q10" s="8" t="str">
+      <c r="Q10" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D10,Q$4&lt;=$E10),"x","")</f>
         <v/>
       </c>
-      <c r="R10" s="8" t="str">
+      <c r="R10" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D10,R$4&lt;=$E10),"x","")</f>
         <v/>
       </c>
-      <c r="S10" s="8" t="str">
+      <c r="S10" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D10,S$4&lt;=$E10),"x","")</f>
         <v/>
       </c>
-      <c r="T10" s="8" t="str">
+      <c r="T10" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D10,T$4&lt;=$E10),"x","")</f>
         <v/>
       </c>
-      <c r="U10" s="8" t="str">
+      <c r="U10" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D10,U$4&lt;=$E10),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="6" t="n">
         <f aca="false">ROUNDUP((E11-D11+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="J11" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="K11" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="M11" s="0" t="s">
+      <c r="M11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="N11" s="8" t="str">
+      <c r="N11" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D11,N$4&lt;=$E11),"x","")</f>
         <v/>
       </c>
-      <c r="O11" s="8" t="str">
+      <c r="O11" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D11,O$4&lt;=$E11),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P11" s="8" t="str">
+      <c r="P11" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D11,P$4&lt;=$E11),"x","")</f>
         <v/>
       </c>
-      <c r="Q11" s="8" t="str">
+      <c r="Q11" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D11,Q$4&lt;=$E11),"x","")</f>
         <v/>
       </c>
-      <c r="R11" s="8" t="str">
+      <c r="R11" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D11,R$4&lt;=$E11),"x","")</f>
         <v/>
       </c>
-      <c r="S11" s="8" t="str">
+      <c r="S11" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D11,S$4&lt;=$E11),"x","")</f>
         <v/>
       </c>
-      <c r="T11" s="8" t="str">
+      <c r="T11" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D11,T$4&lt;=$E11),"x","")</f>
         <v/>
       </c>
-      <c r="U11" s="8" t="str">
+      <c r="U11" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D11,U$4&lt;=$E11),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="6" t="n">
         <f aca="false">ROUNDUP((E12-D12+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="J12" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="K12" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="M12" s="0" t="s">
+      <c r="M12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N12" s="8" t="str">
+      <c r="N12" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D12,N$4&lt;=$E12),"x","")</f>
         <v/>
       </c>
-      <c r="O12" s="8" t="str">
+      <c r="O12" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D12,O$4&lt;=$E12),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P12" s="8" t="str">
+      <c r="P12" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D12,P$4&lt;=$E12),"x","")</f>
         <v/>
       </c>
-      <c r="Q12" s="8" t="str">
+      <c r="Q12" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D12,Q$4&lt;=$E12),"x","")</f>
         <v/>
       </c>
-      <c r="R12" s="8" t="str">
+      <c r="R12" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D12,R$4&lt;=$E12),"x","")</f>
         <v/>
       </c>
-      <c r="S12" s="8" t="str">
+      <c r="S12" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D12,S$4&lt;=$E12),"x","")</f>
         <v/>
       </c>
-      <c r="T12" s="8" t="str">
+      <c r="T12" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D12,T$4&lt;=$E12),"x","")</f>
         <v/>
       </c>
-      <c r="U12" s="8" t="str">
+      <c r="U12" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D12,U$4&lt;=$E12),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="6" t="n">
         <f aca="false">ROUNDUP((E13-D13+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="J13" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="K13" s="3" t="s">
+      <c r="K13" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="M13" s="0" t="s">
+      <c r="M13" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="N13" s="8" t="str">
+      <c r="N13" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D13,N$4&lt;=$E13),"x","")</f>
         <v/>
       </c>
-      <c r="O13" s="8" t="str">
+      <c r="O13" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D13,O$4&lt;=$E13),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P13" s="8" t="str">
+      <c r="P13" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D13,P$4&lt;=$E13),"x","")</f>
         <v/>
       </c>
-      <c r="Q13" s="8" t="str">
+      <c r="Q13" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D13,Q$4&lt;=$E13),"x","")</f>
         <v/>
       </c>
-      <c r="R13" s="8" t="str">
+      <c r="R13" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D13,R$4&lt;=$E13),"x","")</f>
         <v/>
       </c>
-      <c r="S13" s="8" t="str">
+      <c r="S13" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D13,S$4&lt;=$E13),"x","")</f>
         <v/>
       </c>
-      <c r="T13" s="8" t="str">
+      <c r="T13" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D13,T$4&lt;=$E13),"x","")</f>
         <v/>
       </c>
-      <c r="U13" s="8" t="str">
+      <c r="U13" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D13,U$4&lt;=$E13),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="6" t="n">
         <f aca="false">ROUNDUP((E14-D14+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H14" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="J14" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="K14" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="M14" s="0" t="s">
+      <c r="M14" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="N14" s="8" t="str">
+      <c r="N14" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D14,N$4&lt;=$E14),"x","")</f>
         <v/>
       </c>
-      <c r="O14" s="8" t="str">
+      <c r="O14" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D14,O$4&lt;=$E14),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P14" s="8" t="str">
+      <c r="P14" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D14,P$4&lt;=$E14),"x","")</f>
         <v/>
       </c>
-      <c r="Q14" s="8" t="str">
+      <c r="Q14" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D14,Q$4&lt;=$E14),"x","")</f>
         <v/>
       </c>
-      <c r="R14" s="8" t="str">
+      <c r="R14" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D14,R$4&lt;=$E14),"x","")</f>
         <v/>
       </c>
-      <c r="S14" s="8" t="str">
+      <c r="S14" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D14,S$4&lt;=$E14),"x","")</f>
         <v/>
       </c>
-      <c r="T14" s="8" t="str">
+      <c r="T14" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D14,T$4&lt;=$E14),"x","")</f>
         <v/>
       </c>
-      <c r="U14" s="8" t="str">
+      <c r="U14" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D14,U$4&lt;=$E14),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F15" s="5" t="n">
+      <c r="F15" s="6" t="n">
         <f aca="false">ROUNDUP((E15-D15+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H15" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J15" s="3" t="s">
+      <c r="J15" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="K15" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="M15" s="0" t="s">
+      <c r="M15" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="N15" s="8" t="str">
+      <c r="N15" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D15,N$4&lt;=$E15),"x","")</f>
         <v/>
       </c>
-      <c r="O15" s="8" t="str">
+      <c r="O15" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D15,O$4&lt;=$E15),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P15" s="8" t="str">
+      <c r="P15" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D15,P$4&lt;=$E15),"x","")</f>
         <v/>
       </c>
-      <c r="Q15" s="8" t="str">
+      <c r="Q15" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D15,Q$4&lt;=$E15),"x","")</f>
         <v/>
       </c>
-      <c r="R15" s="8" t="str">
+      <c r="R15" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D15,R$4&lt;=$E15),"x","")</f>
         <v/>
       </c>
-      <c r="S15" s="8" t="str">
+      <c r="S15" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D15,S$4&lt;=$E15),"x","")</f>
         <v/>
       </c>
-      <c r="T15" s="8" t="str">
+      <c r="T15" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D15,T$4&lt;=$E15),"x","")</f>
         <v/>
       </c>
-      <c r="U15" s="8" t="str">
+      <c r="U15" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D15,U$4&lt;=$E15),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="6" t="n">
         <f aca="false">ROUNDUP((E16-D16+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="H16" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I16" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="J16" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="K16" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="M16" s="0" t="s">
+      <c r="M16" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="N16" s="8" t="str">
+      <c r="N16" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D16,N$4&lt;=$E16),"x","")</f>
         <v/>
       </c>
-      <c r="O16" s="8" t="str">
+      <c r="O16" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D16,O$4&lt;=$E16),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P16" s="8" t="str">
+      <c r="P16" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D16,P$4&lt;=$E16),"x","")</f>
         <v/>
       </c>
-      <c r="Q16" s="8" t="str">
+      <c r="Q16" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D16,Q$4&lt;=$E16),"x","")</f>
         <v/>
       </c>
-      <c r="R16" s="8" t="str">
+      <c r="R16" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D16,R$4&lt;=$E16),"x","")</f>
         <v/>
       </c>
-      <c r="S16" s="8" t="str">
+      <c r="S16" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D16,S$4&lt;=$E16),"x","")</f>
         <v/>
       </c>
-      <c r="T16" s="8" t="str">
+      <c r="T16" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D16,T$4&lt;=$E16),"x","")</f>
         <v/>
       </c>
-      <c r="U16" s="8" t="str">
+      <c r="U16" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D16,U$4&lt;=$E16),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="5" t="n">
         <v>46208</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="6" t="n">
         <f aca="false">ROUNDUP((E17-D17+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="H17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="I17" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="J17" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="K17" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="M17" s="0" t="s">
+      <c r="M17" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="N17" s="8" t="str">
+      <c r="N17" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D17,N$4&lt;=$E17),"x","")</f>
         <v/>
       </c>
-      <c r="O17" s="8" t="str">
+      <c r="O17" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D17,O$4&lt;=$E17),"x","")</f>
         <v>x</v>
       </c>
-      <c r="P17" s="8" t="str">
+      <c r="P17" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D17,P$4&lt;=$E17),"x","")</f>
         <v/>
       </c>
-      <c r="Q17" s="8" t="str">
+      <c r="Q17" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D17,Q$4&lt;=$E17),"x","")</f>
         <v/>
       </c>
-      <c r="R17" s="8" t="str">
+      <c r="R17" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D17,R$4&lt;=$E17),"x","")</f>
         <v/>
       </c>
-      <c r="S17" s="8" t="str">
+      <c r="S17" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D17,S$4&lt;=$E17),"x","")</f>
         <v/>
       </c>
-      <c r="T17" s="8" t="str">
+      <c r="T17" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D17,T$4&lt;=$E17),"x","")</f>
         <v/>
       </c>
-      <c r="U17" s="8" t="str">
+      <c r="U17" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D17,U$4&lt;=$E17),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="5" t="n">
         <v>46209</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="5" t="n">
         <v>46215</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="6" t="n">
         <f aca="false">ROUNDUP((E18-D18+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="H18" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="I18" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="J18" s="3" t="s">
+      <c r="J18" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="K18" s="3" t="s">
+      <c r="K18" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="M18" s="0" t="s">
+      <c r="M18" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="N18" s="8" t="str">
+      <c r="N18" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D18,N$4&lt;=$E18),"x","")</f>
         <v/>
       </c>
-      <c r="O18" s="8" t="str">
+      <c r="O18" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D18,O$4&lt;=$E18),"x","")</f>
         <v/>
       </c>
-      <c r="P18" s="8" t="str">
+      <c r="P18" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D18,P$4&lt;=$E18),"x","")</f>
         <v>x</v>
       </c>
-      <c r="Q18" s="8" t="str">
+      <c r="Q18" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D18,Q$4&lt;=$E18),"x","")</f>
         <v/>
       </c>
-      <c r="R18" s="8" t="str">
+      <c r="R18" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D18,R$4&lt;=$E18),"x","")</f>
         <v/>
       </c>
-      <c r="S18" s="8" t="str">
+      <c r="S18" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D18,S$4&lt;=$E18),"x","")</f>
         <v/>
       </c>
-      <c r="T18" s="8" t="str">
+      <c r="T18" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D18,T$4&lt;=$E18),"x","")</f>
         <v/>
       </c>
-      <c r="U18" s="8" t="str">
+      <c r="U18" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D18,U$4&lt;=$E18),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="5" t="n">
         <v>46216</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="5" t="n">
         <v>46229</v>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="6" t="n">
         <f aca="false">ROUNDUP((E19-D19+1)/7,0)</f>
         <v>2</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="H19" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="I19" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="J19" s="3" t="s">
+      <c r="J19" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="K19" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="M19" s="0" t="s">
+      <c r="M19" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="N19" s="8" t="str">
+      <c r="N19" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D19,N$4&lt;=$E19),"x","")</f>
         <v/>
       </c>
-      <c r="O19" s="8" t="str">
+      <c r="O19" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D19,O$4&lt;=$E19),"x","")</f>
         <v/>
       </c>
-      <c r="P19" s="8" t="str">
+      <c r="P19" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D19,P$4&lt;=$E19),"x","")</f>
         <v/>
       </c>
-      <c r="Q19" s="8" t="str">
+      <c r="Q19" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D19,Q$4&lt;=$E19),"x","")</f>
         <v>x</v>
       </c>
-      <c r="R19" s="8" t="str">
+      <c r="R19" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D19,R$4&lt;=$E19),"x","")</f>
         <v>x</v>
       </c>
-      <c r="S19" s="8" t="str">
+      <c r="S19" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D19,S$4&lt;=$E19),"x","")</f>
         <v/>
       </c>
-      <c r="T19" s="8" t="str">
+      <c r="T19" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D19,T$4&lt;=$E19),"x","")</f>
         <v/>
       </c>
-      <c r="U19" s="8" t="str">
+      <c r="U19" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D19,U$4&lt;=$E19),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="5" t="n">
         <v>46216</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="5" t="n">
         <v>46222</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="6" t="n">
         <f aca="false">ROUNDUP((E20-D20+1)/7,0)</f>
         <v>1</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H20" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I20" s="3" t="s">
+      <c r="I20" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="J20" s="3" t="s">
+      <c r="J20" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="K20" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="M20" s="0" t="s">
+      <c r="M20" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="N20" s="8" t="str">
+      <c r="N20" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D20,N$4&lt;=$E20),"x","")</f>
         <v/>
       </c>
-      <c r="O20" s="8" t="str">
+      <c r="O20" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D20,O$4&lt;=$E20),"x","")</f>
         <v/>
       </c>
-      <c r="P20" s="8" t="str">
+      <c r="P20" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D20,P$4&lt;=$E20),"x","")</f>
         <v/>
       </c>
-      <c r="Q20" s="8" t="str">
+      <c r="Q20" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D20,Q$4&lt;=$E20),"x","")</f>
         <v>x</v>
       </c>
-      <c r="R20" s="8" t="str">
+      <c r="R20" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D20,R$4&lt;=$E20),"x","")</f>
         <v/>
       </c>
-      <c r="S20" s="8" t="str">
+      <c r="S20" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D20,S$4&lt;=$E20),"x","")</f>
         <v/>
       </c>
-      <c r="T20" s="8" t="str">
+      <c r="T20" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D20,T$4&lt;=$E20),"x","")</f>
         <v/>
       </c>
-      <c r="U20" s="8" t="str">
+      <c r="U20" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D20,U$4&lt;=$E20),"x","")</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="5" t="n">
         <v>46230</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="5" t="n">
         <v>46243</v>
       </c>
-      <c r="F21" s="5" t="n">
+      <c r="F21" s="6" t="n">
         <f aca="false">ROUNDUP((E21-D21+1)/7,0)</f>
         <v>2</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="H21" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="I21" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="J21" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="K21" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="M21" s="0" t="s">
+      <c r="M21" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="N21" s="8" t="str">
+      <c r="N21" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D21,N$4&lt;=$E21),"x","")</f>
         <v/>
       </c>
-      <c r="O21" s="8" t="str">
+      <c r="O21" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D21,O$4&lt;=$E21),"x","")</f>
         <v/>
       </c>
-      <c r="P21" s="8" t="str">
+      <c r="P21" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D21,P$4&lt;=$E21),"x","")</f>
         <v/>
       </c>
-      <c r="Q21" s="8" t="str">
+      <c r="Q21" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D21,Q$4&lt;=$E21),"x","")</f>
         <v/>
       </c>
-      <c r="R21" s="8" t="str">
+      <c r="R21" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D21,R$4&lt;=$E21),"x","")</f>
         <v/>
       </c>
-      <c r="S21" s="8" t="str">
+      <c r="S21" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D21,S$4&lt;=$E21),"x","")</f>
         <v>x</v>
       </c>
-      <c r="T21" s="8" t="str">
+      <c r="T21" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D21,T$4&lt;=$E21),"x","")</f>
         <v>x</v>
       </c>
-      <c r="U21" s="8" t="str">
+      <c r="U21" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D21,U$4&lt;=$E21),"x","")</f>
         <v/>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M22" s="0" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M22" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="N22" s="8" t="str">
+      <c r="N22" s="9" t="str">
         <f aca="false">IF(AND(N$4&gt;=$D22,N$4&lt;=$E22),"x","")</f>
         <v/>
       </c>
-      <c r="O22" s="8" t="str">
+      <c r="O22" s="9" t="str">
         <f aca="false">IF(AND(O$4&gt;=$D22,O$4&lt;=$E22),"x","")</f>
         <v/>
       </c>
-      <c r="P22" s="8" t="str">
+      <c r="P22" s="9" t="str">
         <f aca="false">IF(AND(P$4&gt;=$D22,P$4&lt;=$E22),"x","")</f>
         <v/>
       </c>
-      <c r="Q22" s="8" t="str">
+      <c r="Q22" s="9" t="str">
         <f aca="false">IF(AND(Q$4&gt;=$D22,Q$4&lt;=$E22),"x","")</f>
         <v/>
       </c>
-      <c r="R22" s="8" t="str">
+      <c r="R22" s="9" t="str">
         <f aca="false">IF(AND(R$4&gt;=$D22,R$4&lt;=$E22),"x","")</f>
         <v/>
       </c>
-      <c r="S22" s="8" t="str">
+      <c r="S22" s="9" t="str">
         <f aca="false">IF(AND(S$4&gt;=$D22,S$4&lt;=$E22),"x","")</f>
         <v/>
       </c>
-      <c r="T22" s="8" t="str">
+      <c r="T22" s="9" t="str">
         <f aca="false">IF(AND(T$4&gt;=$D22,T$4&lt;=$E22),"x","")</f>
         <v/>
       </c>
-      <c r="U22" s="8" t="str">
+      <c r="U22" s="9" t="str">
         <f aca="false">IF(AND(U$4&gt;=$D22,U$4&lt;=$E22),"x","")</f>
         <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>46214</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>46214</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="O23" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>46214</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>46214</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="O24" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>46214</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>46214</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O25" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>46214</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>46214</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O26" s="9" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2466,292 +2703,334 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <f aca="false">COUNTA(Cronograma!A4:A26)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <f aca="false">COUNTIF(Cronograma!I4:I26,"Concluido")</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <f aca="false">COUNTIF(Cronograma!I4:I26,"Em andamento")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <f aca="false">COUNTIF(Cronograma!I4:I26,"Nao iniciado")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <f aca="false">COUNTIF(Cronograma!I4:I26,"Bloqueado")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <f aca="false">MAX(Cronograma!E4:E26)</f>
+        <v>46243</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <f aca="false">COUNTA(Cronograma!A4:A21)</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" s="3" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I21,"Concluido")</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" s="3" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I21,"Em andamento")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B7" s="3" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I21,"Nao iniciado")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="B8" s="3" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I21,"Bloqueado")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="B27" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B9" s="4" t="n">
-        <f aca="false">MAX(Cronograma!E4:E21)</f>
-        <v>46243</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="D26" s="3" t="s">
+      <c r="B29" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D29" s="4" t="s">
         <v>55</v>
       </c>
     </row>
@@ -2774,159 +3053,176 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="A1" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>159</v>
+      <c r="A4" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>163</v>
+      <c r="A5" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>163</v>
+      <c r="A6" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>159</v>
+      <c r="A7" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>174</v>
+      <c r="A8" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>178</v>
+      <c r="A9" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>159</v>
+      <c r="A10" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
inicio integracao com waha
</commit_message>
<xml_diff>
--- a/outputs/cronograma-aplicacao-alugueis.xlsx
+++ b/outputs/cronograma-aplicacao-alugueis.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="209">
   <si>
     <t xml:space="preserve">Cronograma de Desenvolvimento - Aplicacao de Alugueis</t>
   </si>
@@ -370,6 +370,18 @@
   </si>
   <si>
     <t xml:space="preserve">Tabela de contratos (admin) ganhou menu de acoes compacto no celular (antes exigia rolagem horizontal por 4 botoes lado a lado). Corrigido botao de remover foto de vistoria que dependia de :hover, invisivel em telas touch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chat de ajuda no painel admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Widget de chat flutuante no painel admin com busca por palavras-chave sobre o manual da aplicacao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baixa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adicionado por solicitacao explicita. Sem IA externa: busca por palavras-chave contra uma base de conhecimento fixa (MANUAL-ADMIN.md / help-content.ts), 100% dentro do Worker atual, nunca consulta o banco de dados (privacidade por construcao). Disponivel apenas no painel admin (dashboard, cadastros, contratos, rateios, integracoes); nao aparece no portal do inquilino nem do recebedor.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo Executivo do Projeto</t>
@@ -1101,7 +1113,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -2671,6 +2683,44 @@
         <v>73</v>
       </c>
       <c r="O26" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="P27" s="9" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2714,7 +2764,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2722,75 +2772,75 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B4" s="4" t="n">
-        <f aca="false">COUNTA(Cronograma!A4:A26)</f>
-        <v>22</v>
+        <f aca="false">COUNTA(Cronograma!A4:A27)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B5" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I26,"Concluido")</f>
-        <v>18</v>
+        <f aca="false">COUNTIF(Cronograma!I4:I27,"Concluido")</f>
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B6" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I26,"Em andamento")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I27,"Em andamento")</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B7" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I26,"Nao iniciado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I27,"Nao iniciado")</f>
         <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B8" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I26,"Bloqueado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I27,"Bloqueado")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B9" s="5" t="n">
-        <f aca="false">MAX(Cronograma!E4:E26)</f>
+        <f aca="false">MAX(Cronograma!E4:E27)</f>
         <v>46243</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>9</v>
@@ -2798,83 +2848,83 @@
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>68</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>7</v>
@@ -2882,13 +2932,13 @@
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>23</v>
@@ -2896,13 +2946,13 @@
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>23</v>
@@ -2910,13 +2960,13 @@
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>150</v>
-      </c>
       <c r="C21" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>23</v>
@@ -2927,10 +2977,10 @@
         <v>61</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>23</v>
@@ -2941,10 +2991,10 @@
         <v>49</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>23</v>
@@ -2955,10 +3005,10 @@
         <v>73</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>23</v>
@@ -2966,13 +3016,13 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>55</v>
@@ -2980,55 +3030,55 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>101</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>55</v>
@@ -3065,7 +3115,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3074,16 +3124,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>9</v>
@@ -3091,138 +3141,138 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>183</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="E10" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>186</v>
-      </c>
       <c r="B11" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajustes cronogramas e layout
</commit_message>
<xml_diff>
--- a/outputs/cronograma-aplicacao-alugueis.xlsx
+++ b/outputs/cronograma-aplicacao-alugueis.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="216">
   <si>
     <t xml:space="preserve">Cronograma de Desenvolvimento - Aplicacao de Alugueis</t>
   </si>
@@ -384,6 +384,30 @@
     <t xml:space="preserve">Adicionado por solicitacao explicita. Sem IA externa: busca por palavras-chave contra uma base de conhecimento fixa (MANUAL-ADMIN.md / help-content.ts), 100% dentro do Worker atual, nunca consulta o banco de dados (privacidade por construcao). Disponivel apenas no painel admin (dashboard, cadastros, contratos, rateios, integracoes); nao aparece no portal do inquilino nem do recebedor.</t>
   </si>
   <si>
+    <t xml:space="preserve">Envio real de lembretes por WhatsApp (WAHA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WAHA self-hosted na AWS enviando lembretes de cobranca via WhatsApp, manual e automatico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desenvolvimento / Infraestrutura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decisao anterior (Cron Trigger + WAHA direto, sem n8n) implementada de fato: WAHA rodando self-hosted em instancia AWS Lightsail (sem HTTPS, decisao explicita, risco aceito). Botao manual "Enviar lembrete WhatsApp" em Cadastros e sweep automatico diario (aviso 5 dias antes, no dia, atraso a cada 3 dias), alem de aviso de pagamento confirmado e de contrato vencendo. Instancia AWS precisou de upgrade de plano (snapshot + plano maior) por instabilidade de memoria no plano inicial de 512MB.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menu lateral fixo em todas as telas admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navegacao (desktop e mobile) presente nas 5 telas do admin, com posicionamento fixo ao rolar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O menu (lateral no desktop, gaveta no mobile) antes so aparecia no Dashboard; agora aparece tambem em Cadastros, Contratos, Rateios e Integracoes, com o item da tela atual destacado. Ambas as versoes (desktop e mobile) ficam fixas (sticky) ao rolar a pagina, em vez de rolar junto com o conteudo.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumo Executivo do Projeto</t>
   </si>
   <si>
@@ -442,9 +466,6 @@
   </si>
   <si>
     <t xml:space="preserve">Define custo e regras de envio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 16</t>
   </si>
   <si>
     <t xml:space="preserve">Definido (revisado 11/07/2026): Cron Trigger da Cloudflare chama o WAHA direto, sem n8n; implementacao do envio pendente</t>
@@ -1113,7 +1134,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -2686,7 +2707,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="102.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
@@ -2721,6 +2742,82 @@
         <v>119</v>
       </c>
       <c r="P27" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="P28" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="P29" s="9" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2764,7 +2861,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2772,75 +2869,75 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B4" s="4" t="n">
-        <f aca="false">COUNTA(Cronograma!A4:A27)</f>
-        <v>23</v>
+        <f aca="false">COUNTA(Cronograma!A4:A29)</f>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B5" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I27,"Concluido")</f>
-        <v>19</v>
+        <f aca="false">COUNTIF(Cronograma!I4:I29,"Concluido")</f>
+        <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B6" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I27,"Em andamento")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I29,"Em andamento")</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="B7" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I27,"Nao iniciado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I29,"Nao iniciado")</f>
         <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B8" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I27,"Bloqueado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I29,"Bloqueado")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B9" s="5" t="n">
-        <f aca="false">MAX(Cronograma!E4:E27)</f>
+        <f aca="false">MAX(Cronograma!E4:E29)</f>
         <v>46243</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>9</v>
@@ -2848,83 +2945,83 @@
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>68</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>7</v>
@@ -2932,13 +3029,13 @@
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>23</v>
@@ -2946,13 +3043,13 @@
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>23</v>
@@ -2960,13 +3057,13 @@
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>23</v>
@@ -2977,10 +3074,10 @@
         <v>61</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>23</v>
@@ -2991,10 +3088,10 @@
         <v>49</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>23</v>
@@ -3005,10 +3102,10 @@
         <v>73</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>23</v>
@@ -3016,13 +3113,13 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>55</v>
@@ -3030,13 +3127,13 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>55</v>
@@ -3047,10 +3144,10 @@
         <v>101</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>55</v>
@@ -3058,13 +3155,13 @@
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>55</v>
@@ -3075,10 +3172,10 @@
         <v>109</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>55</v>
@@ -3115,7 +3212,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3124,16 +3221,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>9</v>
@@ -3141,138 +3238,138 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajustes regra de contrato, permitir o inquilino assinar após todos terem assinado
</commit_message>
<xml_diff>
--- a/outputs/cronograma-aplicacao-alugueis.xlsx
+++ b/outputs/cronograma-aplicacao-alugueis.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="223">
   <si>
     <t xml:space="preserve">Cronograma de Desenvolvimento - Aplicacao de Alugueis</t>
   </si>
@@ -408,6 +408,27 @@
     <t xml:space="preserve">O menu (lateral no desktop, gaveta no mobile) antes so aparecia no Dashboard; agora aparece tambem em Cadastros, Contratos, Rateios e Integracoes, com o item da tela atual destacado. Ambas as versoes (desktop e mobile) ficam fixas (sticky) ao rolar a pagina, em vez de rolar junto com o conteudo.</t>
   </si>
   <si>
+    <t xml:space="preserve">Cadastro de proprietarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novo cadastro de proprietario (dono do imovel), vinculado a pelo menos 1 imovel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adicionado por solicitacao explicita. Novo cadastro 'Proprietario' (admin-only, sem login/portal), distinto de inquilino/imovel/recebedor. Regra: 1 imovel = 1 proprietario (owner_id em properties, nullable); todo proprietario precisa estar vinculado a pelo menos 1 imovel. Tambem confirmado que inquilino e recebedor podem compartilhar o mesmo CPF/CNPJ (ja nao havia restricao no sistema).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testemunhas e ordem de assinatura do contrato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrato com testemunhas selecionaveis (recebedores); inquilino so assina depois que testemunhas e proprietario derem ciencia de assinatura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fases 6 e 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adicionado por solicitacao explicita. Cadastro de contrato ganhou selecao multipla de testemunhas (entre os recebedores cadastrados). Nova tabela contract_witnesses (contract_id, receiver_id, signed_at) e coluna contracts.owner_signed_at. Regra: o inquilino sempre assina por ultimo — isContractReadyForTenantSignature() so libera o link 'Ver contrato e assinatura' no portal do inquilino quando o proprietario do imovel (se houver) e todas as testemunhas do contrato ja tiverem sido marcadas como assinadas pelo admin (novo painel 'Assinaturas' em /cadastros, sem exigir login de testemunhas/proprietario). Pagina /contrato tambem bloqueia o upload da assinatura do inquilino como segunda camada de protecao.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumo Executivo do Projeto</t>
   </si>
   <si>
@@ -468,7 +489,7 @@
     <t xml:space="preserve">Define custo e regras de envio</t>
   </si>
   <si>
-    <t xml:space="preserve">Definido (revisado 11/07/2026): Cron Trigger da Cloudflare chama o WAHA direto, sem n8n; implementacao do envio pendente</t>
+    <t xml:space="preserve">Definido (revisado 12/07/2026): Cron Trigger da Cloudflare chama o WAHA self-hosted (AWS Lightsail) direto, sem n8n; envio real ativo (manual e automatico)</t>
   </si>
   <si>
     <t xml:space="preserve">Armazenamento de PDF assinado</t>
@@ -1134,7 +1155,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U29"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -2745,7 +2766,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="128.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="n">
         <v>24</v>
       </c>
@@ -2783,7 +2804,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="77.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="n">
         <v>25</v>
       </c>
@@ -2818,6 +2839,82 @@
         <v>127</v>
       </c>
       <c r="P29" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="102.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="P30" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J31" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="K31" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="P31" s="9" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2861,7 +2958,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2869,75 +2966,75 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B4" s="4" t="n">
-        <f aca="false">COUNTA(Cronograma!A4:A29)</f>
-        <v>25</v>
+        <f aca="false">COUNTA(Cronograma!A4:A31)</f>
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B5" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I29,"Concluido")</f>
-        <v>21</v>
+        <f aca="false">COUNTIF(Cronograma!I4:I31,"Concluido")</f>
+        <v>23</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B6" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I29,"Em andamento")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I31,"Em andamento")</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="B7" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I29,"Nao iniciado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I31,"Nao iniciado")</f>
         <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="B8" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I29,"Bloqueado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I31,"Bloqueado")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B9" s="5" t="n">
-        <f aca="false">MAX(Cronograma!E4:E29)</f>
+        <f aca="false">MAX(Cronograma!E4:E31)</f>
         <v>46243</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>9</v>
@@ -2945,83 +3042,83 @@
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>68</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>123</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>7</v>
@@ -3029,13 +3126,13 @@
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>23</v>
@@ -3043,13 +3140,13 @@
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>23</v>
@@ -3057,13 +3154,13 @@
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>23</v>
@@ -3074,10 +3171,10 @@
         <v>61</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>23</v>
@@ -3088,10 +3185,10 @@
         <v>49</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>23</v>
@@ -3102,10 +3199,10 @@
         <v>73</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>23</v>
@@ -3113,13 +3210,13 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>55</v>
@@ -3127,13 +3224,13 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>55</v>
@@ -3144,10 +3241,10 @@
         <v>101</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>55</v>
@@ -3155,13 +3252,13 @@
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>55</v>
@@ -3172,10 +3269,10 @@
         <v>109</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>55</v>
@@ -3212,7 +3309,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3221,16 +3318,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>9</v>
@@ -3238,138 +3335,138 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
criado edicao, delete de rateio
</commit_message>
<xml_diff>
--- a/outputs/cronograma-aplicacao-alugueis.xlsx
+++ b/outputs/cronograma-aplicacao-alugueis.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="226">
   <si>
     <t xml:space="preserve">Cronograma de Desenvolvimento - Aplicacao de Alugueis</t>
   </si>
@@ -427,6 +427,15 @@
   </si>
   <si>
     <t xml:space="preserve">Adicionado por solicitacao explicita. Cadastro de contrato ganhou selecao multipla de testemunhas (entre os recebedores cadastrados). Nova tabela contract_witnesses (contract_id, receiver_id, signed_at) e coluna contracts.owner_signed_at. Regra: o inquilino sempre assina por ultimo — isContractReadyForTenantSignature() so libera o link 'Ver contrato e assinatura' no portal do inquilino quando o proprietario do imovel (se houver) e todas as testemunhas do contrato ja tiverem sido marcadas como assinadas pelo admin (novo painel 'Assinaturas' em /cadastros, sem exigir login de testemunhas/proprietario). Pagina /contrato tambem bloqueia o upload da assinatura do inquilino como segunda camada de protecao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edicao e exclusao de rateios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrigir erros operacionais em rateios ja registrados (categoria, valor, imoveis), com reversao automatica do valor ja aplicado nas cobrancas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adicionado por solicitacao explicita (podem ocorrer erros operacionais). Botoes 'Editar' e 'Excluir' por rateio na tela /rateios. updateRateio()/deleteRateio() reaproveitam a logica de calculo de createRateio (extraida para computeAndInsertAllocations): revertem o valor ja aplicado em cobrancas em aberto antes de recalcular/reaplicar (ou de nao reaplicar nada, na exclusao). Nova coluna rateios.split_mode guarda o modo de divisao original para o formulario de edicao. Bloqueado por seguranca se qualquer imovel do rateio ja tiver cobranca paga.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo Executivo do Projeto</t>
@@ -1155,7 +1164,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -2880,7 +2889,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="n">
         <v>27</v>
       </c>
@@ -2915,6 +2924,44 @@
         <v>134</v>
       </c>
       <c r="P31" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>46215</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="P32" s="9" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2958,7 +3005,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2966,75 +3013,75 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B4" s="4" t="n">
-        <f aca="false">COUNTA(Cronograma!A4:A31)</f>
-        <v>27</v>
+        <f aca="false">COUNTA(Cronograma!A4:A32)</f>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B5" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I31,"Concluido")</f>
-        <v>23</v>
+        <f aca="false">COUNTIF(Cronograma!I4:I32,"Concluido")</f>
+        <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B6" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I31,"Em andamento")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I32,"Em andamento")</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B7" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I31,"Nao iniciado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I32,"Nao iniciado")</f>
         <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B8" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I31,"Bloqueado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I32,"Bloqueado")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B9" s="5" t="n">
-        <f aca="false">MAX(Cronograma!E4:E31)</f>
+        <f aca="false">MAX(Cronograma!E4:E32)</f>
         <v>46243</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>9</v>
@@ -3042,83 +3089,83 @@
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>68</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>123</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>7</v>
@@ -3126,13 +3173,13 @@
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>23</v>
@@ -3140,13 +3187,13 @@
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>23</v>
@@ -3154,13 +3201,13 @@
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>23</v>
@@ -3171,10 +3218,10 @@
         <v>61</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>23</v>
@@ -3185,10 +3232,10 @@
         <v>49</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>23</v>
@@ -3199,10 +3246,10 @@
         <v>73</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>23</v>
@@ -3210,13 +3257,13 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>55</v>
@@ -3224,13 +3271,13 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>55</v>
@@ -3241,10 +3288,10 @@
         <v>101</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>55</v>
@@ -3252,13 +3299,13 @@
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>55</v>
@@ -3269,10 +3316,10 @@
         <v>109</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>55</v>
@@ -3309,7 +3356,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3318,16 +3365,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>9</v>
@@ -3335,138 +3382,138 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>200</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajustes estruturais, refatoracao, separacao cadastros
</commit_message>
<xml_diff>
--- a/outputs/cronograma-aplicacao-alugueis.xlsx
+++ b/outputs/cronograma-aplicacao-alugueis.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="238">
   <si>
     <t xml:space="preserve">Cronograma de Desenvolvimento - Aplicacao de Alugueis</t>
   </si>
@@ -438,6 +438,33 @@
     <t xml:space="preserve">Adicionado por solicitacao explicita (podem ocorrer erros operacionais). Botoes 'Editar' e 'Excluir' por rateio na tela /rateios. updateRateio()/deleteRateio() reaproveitam a logica de calculo de createRateio (extraida para computeAndInsertAllocations): revertem o valor ja aplicado em cobrancas em aberto antes de recalcular/reaplicar (ou de nao reaplicar nada, na exclusao). Nova coluna rateios.split_mode guarda o modo de divisao original para o formulario de edicao. Bloqueado por seguranca se qualquer imovel do rateio ja tiver cobranca paga.</t>
   </si>
   <si>
+    <t xml:space="preserve">Refatoracao e qualidade de codigo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deduplicacao de helpers das rotas de API, modulos financeiros puros com testes unitarios, divisao do CadastroWorkspace (1.670 -&gt; ~870 linhas), IDs via crypto.randomUUID, schema Drizzle sincronizado com o DDL runtime, limpeza de arquivos de trabalho do repositorio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fases 2 e 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Originado da auditoria de codigo de 13/07/2026. Novos modulos: app/lib/api-helpers.ts (getErrorMessage/errorStatus/requiredString/escapeHtml antes copiados em 27 rotas), app/lib/finance.ts (multa/juros e divisao de rateio em centavos) e app/lib/billing-cycle.ts (datas do ciclo de cobranca) — ambos puros e cobertos por 16 testes (npm test, runner nativo do Node, sem dependencia nova). CadastroWorkspace.tsx dividido em ui.tsx, ManagementPanel.tsx, checkbox-lists.tsx, contract-components.tsx, ContractsSection.tsx e support.ts. db/schema.ts agora espelha o schema real provisionado em runtime (tabelas reminders/audit_logs mortas removidas). Corrigidos 5 erros de tipo pre-existentes (cast de env e BodyInit do recibo PDF).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardening de seguranca (pendente)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPS entre Cloudflare e WAHA, remover senhas seed do codigo, indice UNIQUE em payments.external_id, rate limiting no login, validacao fail-closed do webhook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fase 29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apontado na auditoria de 13/07/2026, ainda nao implementado: (1) WAHA em HTTP puro expoe WAHA_API_KEY e telefones em transito; (2) senha do admin seed (TrocarSenha!2026) e dos usuarios demo esta hardcoded no repositorio — trocar em producao e mover para secret; (3) recordApprovedPayment e check-then-insert sem UNIQUE em payments.external_id (webhooks simultaneos podem duplicar pagamento); (4) login sem rate limiting; (5) validateWebhookSignature retorna true quando MP_WEBHOOK_SECRET nao esta configurado (fail-open).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumo Executivo do Projeto</t>
   </si>
   <si>
@@ -654,45 +681,45 @@
     <t xml:space="preserve">Cobranca indevida ou perda financeira</t>
   </si>
   <si>
-    <t xml:space="preserve">Adicionar testes automatizados para multa, juros, carencia e abonos</t>
+    <t xml:space="preserve">Logica de multa/juros extraida para modulo puro (app/lib/finance.ts) e coberta por testes unitarios (npm test): multa fixa, juros pro rata dia, carencia, cobranca paga e divisao de rateio em centavos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mensagens WhatsApp duplicadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiencia ruim para o inquilino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controlar envio por cobranca, evento e data quando a integracao Cron Trigger + WAHA (sem n8n, decisao de 11/07/2026) for implementada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aberto (fase nao iniciada)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Armazenamento de documentos sensiveis (contratos assinados)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risco de LGPD e seguranca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDF assinado armazenado no R2 (fora do banco); revisar politica de retencao e controle de acesso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitigado parcialmente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ausencia de teste de ponta a ponta ao vivo da aplicacao publicada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bugs de integracao podem passar despercebidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realizar bateria de testes manuais (ou via navegador) cobrindo os fluxos criticos antes do lancamento</t>
   </si>
   <si>
     <t xml:space="preserve">Aberto</t>
   </si>
   <si>
-    <t xml:space="preserve">Mensagens WhatsApp duplicadas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiencia ruim para o inquilino</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controlar envio por cobranca, evento e data quando a integracao Cron Trigger + WAHA (sem n8n, decisao de 11/07/2026) for implementada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aberto (fase nao iniciada)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Armazenamento de documentos sensiveis (contratos assinados)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risco de LGPD e seguranca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PDF assinado armazenado no R2 (fora do banco); revisar politica de retencao e controle de acesso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitigado parcialmente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ausencia de teste de ponta a ponta ao vivo da aplicacao publicada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bugs de integracao podem passar despercebidos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Realizar bateria de testes manuais (ou via navegador) cobrindo os fluxos criticos antes do lancamento</t>
-  </si>
-  <si>
     <t xml:space="preserve">Apenas uma transacao Pix real (R$1) foi validada</t>
   </si>
   <si>
@@ -700,6 +727,15 @@
   </si>
   <si>
     <t xml:space="preserve">Realizar mais alguns testes reais de baixo valor cobrindo expiracao e falha antes do uso pleno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credenciais seed no codigo e WAHA sem HTTPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acesso admin indevido (senha seed conhecida no repositorio) e vazamento de API key/telefones em transito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trocar a senha do admin em producao, mover seeds para secrets e colocar o WAHA atras de HTTPS (fase 30 do cronograma).</t>
   </si>
 </sst>
 </file>
@@ -1164,7 +1200,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -2927,7 +2963,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="128.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
         <v>28</v>
       </c>
@@ -2963,6 +2999,72 @@
       </c>
       <c r="P32" s="9" t="s">
         <v>104</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>46216</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E34" s="5"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="J34" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -3005,7 +3107,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3013,60 +3115,60 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="B4" s="4" t="n">
-        <f aca="false">COUNTA(Cronograma!A4:A32)</f>
-        <v>28</v>
+        <f aca="false">COUNTA(Cronograma!A4:A34)</f>
+        <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="B5" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I32,"Concluido")</f>
-        <v>24</v>
+        <f aca="false">COUNTIF(Cronograma!I4:I34,"Concluido")</f>
+        <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="B6" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I32,"Em andamento")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I34,"Em andamento")</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="B7" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I32,"Nao iniciado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I34,"Nao iniciado")</f>
         <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="B8" s="4" t="n">
-        <f aca="false">COUNTIF(Cronograma!I4:I32,"Bloqueado")</f>
+        <f aca="false">COUNTIF(Cronograma!I4:I34,"Bloqueado")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">MAX(Cronograma!E4:E32)</f>
@@ -3075,13 +3177,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>9</v>
@@ -3089,83 +3191,83 @@
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>68</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>123</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>7</v>
@@ -3173,13 +3275,13 @@
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>23</v>
@@ -3187,13 +3289,13 @@
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>23</v>
@@ -3201,13 +3303,13 @@
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>23</v>
@@ -3218,10 +3320,10 @@
         <v>61</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>23</v>
@@ -3232,10 +3334,10 @@
         <v>49</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>23</v>
@@ -3246,10 +3348,10 @@
         <v>73</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>23</v>
@@ -3257,13 +3359,13 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>55</v>
@@ -3271,13 +3373,13 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>55</v>
@@ -3288,10 +3390,10 @@
         <v>101</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>55</v>
@@ -3299,13 +3401,13 @@
     </row>
     <row r="28" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>55</v>
@@ -3316,10 +3418,10 @@
         <v>109</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>55</v>
@@ -3344,7 +3446,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -3356,7 +3458,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3365,16 +3467,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>9</v>
@@ -3382,138 +3484,155 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>209</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>211</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>211</v>
+        <v>231</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>